<commit_message>
Add data for 2026-09-04
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-ytd.xlsx
+++ b/output/cta-index-crime-ytd.xlsx
@@ -9,30 +9,30 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Lake View" sheetId="3" r:id="rId3"/>
-    <sheet name="North Lawndale" sheetId="4" r:id="rId4"/>
-    <sheet name="Hyde Park" sheetId="5" r:id="rId5"/>
-    <sheet name="Grand Boulevard" sheetId="6" r:id="rId6"/>
-    <sheet name="Avondale" sheetId="7" r:id="rId7"/>
-    <sheet name="West Town" sheetId="8" r:id="rId8"/>
-    <sheet name="West Loop" sheetId="9" r:id="rId9"/>
-    <sheet name="Douglas" sheetId="10" r:id="rId10"/>
-    <sheet name="South Shore" sheetId="11" r:id="rId11"/>
-    <sheet name="Loop" sheetId="12" r:id="rId12"/>
-    <sheet name="Chatham" sheetId="13" r:id="rId13"/>
-    <sheet name="Norwood Park" sheetId="14" r:id="rId14"/>
-    <sheet name="Washington Park" sheetId="15" r:id="rId15"/>
-    <sheet name="Fuller Park" sheetId="16" r:id="rId16"/>
-    <sheet name="Englewood" sheetId="17" r:id="rId17"/>
-    <sheet name="Greektown" sheetId="18" r:id="rId18"/>
-    <sheet name="Rogers Park" sheetId="19" r:id="rId19"/>
-    <sheet name="Austin" sheetId="20" r:id="rId20"/>
-    <sheet name="River North" sheetId="21" r:id="rId21"/>
-    <sheet name="Garfield Park" sheetId="22" r:id="rId22"/>
-    <sheet name="Lincoln Park" sheetId="23" r:id="rId23"/>
-    <sheet name="Edgewater" sheetId="24" r:id="rId24"/>
-    <sheet name="Little Italy, UIC" sheetId="25" r:id="rId25"/>
-    <sheet name="Uptown" sheetId="26" r:id="rId26"/>
+    <sheet name="Uptown" sheetId="3" r:id="rId3"/>
+    <sheet name="Lake View" sheetId="4" r:id="rId4"/>
+    <sheet name="North Lawndale" sheetId="5" r:id="rId5"/>
+    <sheet name="Hyde Park" sheetId="6" r:id="rId6"/>
+    <sheet name="Grand Boulevard" sheetId="7" r:id="rId7"/>
+    <sheet name="Avondale" sheetId="8" r:id="rId8"/>
+    <sheet name="West Town" sheetId="9" r:id="rId9"/>
+    <sheet name="West Loop" sheetId="10" r:id="rId10"/>
+    <sheet name="Douglas" sheetId="11" r:id="rId11"/>
+    <sheet name="South Shore" sheetId="12" r:id="rId12"/>
+    <sheet name="Loop" sheetId="13" r:id="rId13"/>
+    <sheet name="Chatham" sheetId="14" r:id="rId14"/>
+    <sheet name="Norwood Park" sheetId="15" r:id="rId15"/>
+    <sheet name="Washington Park" sheetId="16" r:id="rId16"/>
+    <sheet name="Fuller Park" sheetId="17" r:id="rId17"/>
+    <sheet name="Englewood" sheetId="18" r:id="rId18"/>
+    <sheet name="Greektown" sheetId="19" r:id="rId19"/>
+    <sheet name="Rogers Park" sheetId="20" r:id="rId20"/>
+    <sheet name="Austin" sheetId="21" r:id="rId21"/>
+    <sheet name="River North" sheetId="22" r:id="rId22"/>
+    <sheet name="Garfield Park" sheetId="23" r:id="rId23"/>
+    <sheet name="Lincoln Park" sheetId="24" r:id="rId24"/>
+    <sheet name="Edgewater" sheetId="25" r:id="rId25"/>
+    <sheet name="Little Italy, UIC" sheetId="26" r:id="rId26"/>
     <sheet name="Albany Park" sheetId="27" r:id="rId27"/>
     <sheet name="Grand Crossing" sheetId="28" r:id="rId28"/>
     <sheet name="Washington Heights" sheetId="29" r:id="rId29"/>
@@ -946,7 +946,7 @@
         <v>170</v>
       </c>
       <c r="M3">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1232,7 +1232,7 @@
         <v>1086</v>
       </c>
       <c r="M11">
-        <v>790</v>
+        <v>791</v>
       </c>
     </row>
   </sheetData>
@@ -1241,6 +1241,283 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>7</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <v>4</v>
+      </c>
+      <c r="L7">
+        <v>4</v>
+      </c>
+      <c r="M7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <v>25</v>
+      </c>
+      <c r="E8">
+        <v>19</v>
+      </c>
+      <c r="F8">
+        <v>33</v>
+      </c>
+      <c r="G8">
+        <v>14</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8">
+        <v>17</v>
+      </c>
+      <c r="J8">
+        <v>16</v>
+      </c>
+      <c r="K8">
+        <v>11</v>
+      </c>
+      <c r="L8">
+        <v>9</v>
+      </c>
+      <c r="M8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>32</v>
+      </c>
+      <c r="E9">
+        <v>23</v>
+      </c>
+      <c r="F9">
+        <v>40</v>
+      </c>
+      <c r="G9">
+        <v>24</v>
+      </c>
+      <c r="H9">
+        <v>16</v>
+      </c>
+      <c r="I9">
+        <v>26</v>
+      </c>
+      <c r="J9">
+        <v>19</v>
+      </c>
+      <c r="K9">
+        <v>18</v>
+      </c>
+      <c r="L9">
+        <v>17</v>
+      </c>
+      <c r="M9">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1479,7 +1756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1732,7 +2009,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2074,7 +2351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2354,222 +2631,6 @@
       </c>
       <c r="M8">
         <v>17</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>10</v>
-      </c>
-      <c r="C6">
-        <v>8</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>12</v>
-      </c>
-      <c r="F6">
-        <v>12</v>
-      </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>8</v>
-      </c>
-      <c r="D7">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>12</v>
-      </c>
-      <c r="F7">
-        <v>13</v>
-      </c>
-      <c r="G7">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <v>6</v>
-      </c>
-      <c r="I7">
-        <v>3</v>
-      </c>
-      <c r="J7">
-        <v>2</v>
-      </c>
-      <c r="K7">
-        <v>6</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2642,17 +2703,8 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
+      <c r="K2">
+        <v>1</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -2665,42 +2717,30 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
+      <c r="F3">
+        <v>1</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L4">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
@@ -2708,32 +2748,14 @@
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
       <c r="D5">
-        <v>7</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -2742,7 +2764,7 @@
         <v>1</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2750,40 +2772,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C6">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>12</v>
+      </c>
+      <c r="F6">
+        <v>12</v>
+      </c>
+      <c r="G6">
         <v>7</v>
       </c>
-      <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
       <c r="H6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2791,40 +2813,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D7">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E7">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F7">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G7">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H7">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I7">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K7">
+        <v>6</v>
+      </c>
+      <c r="L7">
         <v>7</v>
       </c>
-      <c r="L7">
-        <v>6</v>
-      </c>
       <c r="M7">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2833,6 +2855,261 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>8</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>15</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>9</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>18</v>
+      </c>
+      <c r="C7">
+        <v>23</v>
+      </c>
+      <c r="D7">
+        <v>16</v>
+      </c>
+      <c r="E7">
+        <v>14</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>9</v>
+      </c>
+      <c r="I7">
+        <v>13</v>
+      </c>
+      <c r="J7">
+        <v>9</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>6</v>
+      </c>
+      <c r="M7">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3106,7 +3383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3413,7 +3690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3610,293 +3887,6 @@
       </c>
       <c r="M7">
         <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>6</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>7</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6">
-        <v>13</v>
-      </c>
-      <c r="G6">
-        <v>5</v>
-      </c>
-      <c r="H6">
-        <v>10</v>
-      </c>
-      <c r="I6">
-        <v>11</v>
-      </c>
-      <c r="J6">
-        <v>9</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
-      <c r="L6">
-        <v>9</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>31</v>
-      </c>
-      <c r="C7">
-        <v>40</v>
-      </c>
-      <c r="D7">
-        <v>32</v>
-      </c>
-      <c r="E7">
-        <v>59</v>
-      </c>
-      <c r="F7">
-        <v>29</v>
-      </c>
-      <c r="G7">
-        <v>22</v>
-      </c>
-      <c r="H7">
-        <v>17</v>
-      </c>
-      <c r="I7">
-        <v>18</v>
-      </c>
-      <c r="J7">
-        <v>21</v>
-      </c>
-      <c r="K7">
-        <v>20</v>
-      </c>
-      <c r="L7">
-        <v>22</v>
-      </c>
-      <c r="M7">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>33</v>
-      </c>
-      <c r="C8">
-        <v>52</v>
-      </c>
-      <c r="D8">
-        <v>42</v>
-      </c>
-      <c r="E8">
-        <v>73</v>
-      </c>
-      <c r="F8">
-        <v>44</v>
-      </c>
-      <c r="G8">
-        <v>32</v>
-      </c>
-      <c r="H8">
-        <v>30</v>
-      </c>
-      <c r="I8">
-        <v>35</v>
-      </c>
-      <c r="J8">
-        <v>32</v>
-      </c>
-      <c r="K8">
-        <v>39</v>
-      </c>
-      <c r="L8">
-        <v>38</v>
-      </c>
-      <c r="M8">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -7083,7 +7073,7 @@
         <v>22</v>
       </c>
       <c r="M87">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -7557,7 +7547,7 @@
         <v>1086</v>
       </c>
       <c r="M99">
-        <v>790</v>
+        <v>791</v>
       </c>
     </row>
   </sheetData>
@@ -7667,6 +7657,293 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>6</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>9</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
+        <v>13</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>11</v>
+      </c>
+      <c r="J6">
+        <v>9</v>
+      </c>
+      <c r="K6">
+        <v>9</v>
+      </c>
+      <c r="L6">
+        <v>9</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>31</v>
+      </c>
+      <c r="C7">
+        <v>40</v>
+      </c>
+      <c r="D7">
+        <v>32</v>
+      </c>
+      <c r="E7">
+        <v>59</v>
+      </c>
+      <c r="F7">
+        <v>29</v>
+      </c>
+      <c r="G7">
+        <v>22</v>
+      </c>
+      <c r="H7">
+        <v>17</v>
+      </c>
+      <c r="I7">
+        <v>18</v>
+      </c>
+      <c r="J7">
+        <v>21</v>
+      </c>
+      <c r="K7">
+        <v>20</v>
+      </c>
+      <c r="L7">
+        <v>22</v>
+      </c>
+      <c r="M7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>33</v>
+      </c>
+      <c r="C8">
+        <v>52</v>
+      </c>
+      <c r="D8">
+        <v>42</v>
+      </c>
+      <c r="E8">
+        <v>73</v>
+      </c>
+      <c r="F8">
+        <v>44</v>
+      </c>
+      <c r="G8">
+        <v>32</v>
+      </c>
+      <c r="H8">
+        <v>30</v>
+      </c>
+      <c r="I8">
+        <v>35</v>
+      </c>
+      <c r="J8">
+        <v>32</v>
+      </c>
+      <c r="K8">
+        <v>39</v>
+      </c>
+      <c r="L8">
+        <v>38</v>
+      </c>
+      <c r="M8">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -7975,7 +8252,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8239,7 +8516,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8543,7 +8820,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8768,7 +9045,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9031,7 +9308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9297,286 +9574,6 @@
       </c>
       <c r="M7">
         <v>18</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>5</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-      <c r="E7">
-        <v>3</v>
-      </c>
-      <c r="F7">
-        <v>4</v>
-      </c>
-      <c r="G7">
-        <v>13</v>
-      </c>
-      <c r="H7">
-        <v>6</v>
-      </c>
-      <c r="I7">
-        <v>4</v>
-      </c>
-      <c r="J7">
-        <v>4</v>
-      </c>
-      <c r="K7">
-        <v>5</v>
-      </c>
-      <c r="L7">
-        <v>6</v>
-      </c>
-      <c r="M7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>19</v>
-      </c>
-      <c r="C8">
-        <v>21</v>
-      </c>
-      <c r="D8">
-        <v>13</v>
-      </c>
-      <c r="E8">
-        <v>16</v>
-      </c>
-      <c r="F8">
-        <v>13</v>
-      </c>
-      <c r="G8">
-        <v>13</v>
-      </c>
-      <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>10</v>
-      </c>
-      <c r="J8">
-        <v>10</v>
-      </c>
-      <c r="K8">
-        <v>8</v>
-      </c>
-      <c r="L8">
-        <v>12</v>
-      </c>
-      <c r="M8">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>25</v>
-      </c>
-      <c r="C9">
-        <v>29</v>
-      </c>
-      <c r="D9">
-        <v>15</v>
-      </c>
-      <c r="E9">
-        <v>24</v>
-      </c>
-      <c r="F9">
-        <v>20</v>
-      </c>
-      <c r="G9">
-        <v>32</v>
-      </c>
-      <c r="H9">
-        <v>20</v>
-      </c>
-      <c r="I9">
-        <v>18</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>21</v>
-      </c>
-      <c r="L9">
-        <v>22</v>
-      </c>
-      <c r="M9">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -10349,7 +10346,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -10413,82 +10410,76 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>3</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>4</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="E4">
         <v>1</v>
       </c>
     </row>
@@ -10496,143 +10487,136 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
+      <c r="B5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6">
-        <v>10</v>
-      </c>
-      <c r="D6">
-        <v>7</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
-      <c r="F6">
-        <v>8</v>
-      </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>10</v>
-      </c>
-      <c r="I6">
-        <v>16</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C7">
-        <v>35</v>
-      </c>
-      <c r="D7">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E7">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="G7">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="I7">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="J7">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="L7">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M7">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>19</v>
+      </c>
+      <c r="C8">
+        <v>21</v>
+      </c>
+      <c r="D8">
+        <v>13</v>
+      </c>
+      <c r="E8">
+        <v>16</v>
+      </c>
+      <c r="F8">
+        <v>13</v>
+      </c>
+      <c r="G8">
+        <v>13</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
         <v>10</v>
       </c>
-      <c r="B8">
-        <v>34</v>
-      </c>
-      <c r="C8">
-        <v>54</v>
-      </c>
-      <c r="D8">
-        <v>38</v>
-      </c>
-      <c r="E8">
-        <v>49</v>
-      </c>
-      <c r="F8">
-        <v>54</v>
-      </c>
-      <c r="G8">
-        <v>47</v>
-      </c>
-      <c r="H8">
+      <c r="J8">
+        <v>10</v>
+      </c>
+      <c r="K8">
+        <v>8</v>
+      </c>
+      <c r="L8">
+        <v>12</v>
+      </c>
+      <c r="M8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>25</v>
+      </c>
+      <c r="C9">
         <v>29</v>
       </c>
-      <c r="I8">
-        <v>39</v>
-      </c>
-      <c r="J8">
-        <v>28</v>
-      </c>
-      <c r="K8">
-        <v>27</v>
-      </c>
-      <c r="L8">
-        <v>29</v>
-      </c>
-      <c r="M8">
-        <v>25</v>
+      <c r="D9">
+        <v>15</v>
+      </c>
+      <c r="E9">
+        <v>24</v>
+      </c>
+      <c r="F9">
+        <v>20</v>
+      </c>
+      <c r="G9">
+        <v>32</v>
+      </c>
+      <c r="H9">
+        <v>20</v>
+      </c>
+      <c r="I9">
+        <v>18</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>21</v>
+      </c>
+      <c r="L9">
+        <v>22</v>
+      </c>
+      <c r="M9">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -12915,26 +12899,20 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -12943,13 +12921,13 @@
         <v>1</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L2">
         <v>3</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -12957,9 +12935,12 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
@@ -12969,35 +12950,32 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="I4">
+        <v>4</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
@@ -13005,49 +12983,61 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
       <c r="H5">
         <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>10</v>
       </c>
-      <c r="C6">
-        <v>12</v>
-      </c>
       <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>7</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
         <v>16</v>
       </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6">
-        <v>21</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>5</v>
-      </c>
-      <c r="I6">
-        <v>14</v>
-      </c>
       <c r="J6">
         <v>2</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6">
         <v>5</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -13055,40 +13045,40 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D7">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="F7">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="G7">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="H7">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I7">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="J7">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="K7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="M7">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -13096,40 +13086,40 @@
         <v>10</v>
       </c>
       <c r="B8">
+        <v>34</v>
+      </c>
+      <c r="C8">
+        <v>54</v>
+      </c>
+      <c r="D8">
+        <v>38</v>
+      </c>
+      <c r="E8">
+        <v>49</v>
+      </c>
+      <c r="F8">
+        <v>54</v>
+      </c>
+      <c r="G8">
+        <v>47</v>
+      </c>
+      <c r="H8">
+        <v>29</v>
+      </c>
+      <c r="I8">
+        <v>39</v>
+      </c>
+      <c r="J8">
+        <v>28</v>
+      </c>
+      <c r="K8">
         <v>27</v>
       </c>
-      <c r="C8">
-        <v>37</v>
-      </c>
-      <c r="D8">
-        <v>40</v>
-      </c>
-      <c r="E8">
-        <v>30</v>
-      </c>
-      <c r="F8">
-        <v>52</v>
-      </c>
-      <c r="G8">
-        <v>37</v>
-      </c>
-      <c r="H8">
-        <v>15</v>
-      </c>
-      <c r="I8">
-        <v>27</v>
-      </c>
-      <c r="J8">
-        <v>8</v>
-      </c>
-      <c r="K8">
-        <v>19</v>
-      </c>
       <c r="L8">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="M8">
-        <v>11</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -15324,10 +15314,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -15387,10 +15377,40 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
       <c r="H2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -15398,143 +15418,180 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
       <c r="E3">
         <v>1</v>
       </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="H4">
         <v>1</v>
       </c>
       <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>5</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>7</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>6</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>3</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
         <v>10</v>
       </c>
-      <c r="B6">
-        <v>4</v>
-      </c>
       <c r="C6">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>21</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>14</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F6">
-        <v>6</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
+      <c r="B7">
+        <v>14</v>
+      </c>
+      <c r="C7">
+        <v>23</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>28</v>
+      </c>
+      <c r="G7">
+        <v>22</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
         <v>7</v>
       </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-      <c r="J6">
-        <v>12</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
+      <c r="J7">
+        <v>4</v>
+      </c>
+      <c r="K7">
+        <v>10</v>
+      </c>
+      <c r="L7">
+        <v>4</v>
+      </c>
+      <c r="M7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>40</v>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>52</v>
+      </c>
+      <c r="G8">
+        <v>37</v>
+      </c>
+      <c r="H8">
+        <v>15</v>
+      </c>
+      <c r="I8">
+        <v>27</v>
+      </c>
+      <c r="J8">
+        <v>8</v>
+      </c>
+      <c r="K8">
+        <v>19</v>
+      </c>
+      <c r="L8">
+        <v>16</v>
+      </c>
+      <c r="M8">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -17706,7 +17763,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -17769,183 +17826,154 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
       <c r="H2">
         <v>1</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
+      <c r="I2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
       </c>
       <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>5</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>7</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
         <v>6</v>
       </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
       <c r="K5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
         <v>9</v>
       </c>
-      <c r="B6">
-        <v>9</v>
-      </c>
-      <c r="C6">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>8</v>
-      </c>
-      <c r="E6">
-        <v>13</v>
-      </c>
       <c r="F6">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
         <v>7</v>
       </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-      <c r="H6">
-        <v>3</v>
-      </c>
       <c r="I6">
         <v>5</v>
       </c>
       <c r="J6">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>14</v>
-      </c>
-      <c r="C7">
-        <v>16</v>
-      </c>
-      <c r="D7">
-        <v>14</v>
-      </c>
-      <c r="E7">
-        <v>18</v>
-      </c>
-      <c r="F7">
-        <v>11</v>
-      </c>
-      <c r="G7">
-        <v>13</v>
-      </c>
-      <c r="H7">
-        <v>7</v>
-      </c>
-      <c r="I7">
-        <v>9</v>
-      </c>
-      <c r="J7">
-        <v>12</v>
-      </c>
-      <c r="K7">
-        <v>11</v>
-      </c>
-      <c r="L7">
-        <v>14</v>
-      </c>
-      <c r="M7">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -19572,7 +19600,7 @@
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -19632,23 +19660,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
         <v>1</v>
       </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
       <c r="J2">
         <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
       </c>
       <c r="M2">
         <v>2</v>
@@ -19658,8 +19689,8 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E3">
-        <v>1</v>
+      <c r="B3">
+        <v>2</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -19667,21 +19698,24 @@
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="J3">
-        <v>2</v>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K4">
+        <v>6</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
@@ -19690,34 +19724,37 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H5">
         <v>2</v>
       </c>
       <c r="I5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>3</v>
       </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
       <c r="L5">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -19725,40 +19762,40 @@
         <v>9</v>
       </c>
       <c r="B6">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>9</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>13</v>
+      </c>
+      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="G6">
+        <v>8</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>8</v>
+      </c>
+      <c r="K6">
         <v>6</v>
       </c>
-      <c r="C6">
-        <v>5</v>
-      </c>
-      <c r="D6">
-        <v>24</v>
-      </c>
-      <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>7</v>
-      </c>
-      <c r="J6">
-        <v>7</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
       <c r="L6">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -19766,40 +19803,40 @@
         <v>10</v>
       </c>
       <c r="B7">
+        <v>14</v>
+      </c>
+      <c r="C7">
+        <v>16</v>
+      </c>
+      <c r="D7">
+        <v>14</v>
+      </c>
+      <c r="E7">
+        <v>18</v>
+      </c>
+      <c r="F7">
+        <v>11</v>
+      </c>
+      <c r="G7">
+        <v>13</v>
+      </c>
+      <c r="H7">
+        <v>7</v>
+      </c>
+      <c r="I7">
         <v>9</v>
       </c>
-      <c r="C7">
-        <v>7</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>13</v>
-      </c>
-      <c r="F7">
+      <c r="J7">
+        <v>12</v>
+      </c>
+      <c r="K7">
+        <v>11</v>
+      </c>
+      <c r="L7">
         <v>14</v>
       </c>
-      <c r="G7">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>11</v>
-      </c>
-      <c r="J7">
-        <v>13</v>
-      </c>
-      <c r="K7">
-        <v>10</v>
-      </c>
-      <c r="L7">
-        <v>15</v>
-      </c>
       <c r="M7">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -21776,8 +21813,8 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="D2">
-        <v>3</v>
+      <c r="C2">
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -21786,52 +21823,43 @@
         <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
+      <c r="J3">
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
@@ -21843,37 +21871,31 @@
         <v>2</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L5">
-        <v>4</v>
-      </c>
-      <c r="M5">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -21881,40 +21903,40 @@
         <v>9</v>
       </c>
       <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>24</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="I6">
         <v>7</v>
       </c>
-      <c r="C6">
-        <v>18</v>
-      </c>
-      <c r="D6">
-        <v>29</v>
-      </c>
-      <c r="E6">
-        <v>60</v>
-      </c>
-      <c r="F6">
-        <v>43</v>
-      </c>
-      <c r="G6">
+      <c r="J6">
+        <v>7</v>
+      </c>
+      <c r="K6">
         <v>9</v>
       </c>
-      <c r="H6">
-        <v>5</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
-      <c r="J6">
-        <v>4</v>
-      </c>
-      <c r="K6">
+      <c r="L6">
         <v>12</v>
       </c>
-      <c r="L6">
-        <v>9</v>
-      </c>
       <c r="M6">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -21922,40 +21944,40 @@
         <v>10</v>
       </c>
       <c r="B7">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>14</v>
+      </c>
+      <c r="G7">
+        <v>8</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>11</v>
+      </c>
+      <c r="J7">
+        <v>13</v>
+      </c>
+      <c r="K7">
         <v>10</v>
       </c>
-      <c r="C7">
-        <v>22</v>
-      </c>
-      <c r="D7">
-        <v>40</v>
-      </c>
-      <c r="E7">
-        <v>65</v>
-      </c>
-      <c r="F7">
-        <v>49</v>
-      </c>
-      <c r="G7">
-        <v>12</v>
-      </c>
-      <c r="H7">
-        <v>11</v>
-      </c>
-      <c r="I7">
+      <c r="L7">
         <v>15</v>
       </c>
-      <c r="J7">
-        <v>8</v>
-      </c>
-      <c r="K7">
-        <v>19</v>
-      </c>
-      <c r="L7">
-        <v>20</v>
-      </c>
       <c r="M7">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -23467,7 +23489,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -23533,207 +23555,185 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="G2">
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
         <v>1</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
       <c r="K2">
         <v>2</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
         <v>1</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="L4">
+      <c r="J4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
         <v>6</v>
       </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
       <c r="I5">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
         <v>7</v>
       </c>
+      <c r="C6">
+        <v>18</v>
+      </c>
       <c r="D6">
-        <v>1</v>
+        <v>29</v>
+      </c>
+      <c r="E6">
+        <v>60</v>
+      </c>
+      <c r="F6">
+        <v>43</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>8</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+      <c r="K6">
+        <v>12</v>
+      </c>
+      <c r="L6">
+        <v>9</v>
+      </c>
+      <c r="M6">
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>40</v>
+      </c>
+      <c r="E7">
+        <v>65</v>
+      </c>
+      <c r="F7">
+        <v>49</v>
+      </c>
+      <c r="G7">
+        <v>12</v>
+      </c>
+      <c r="H7">
+        <v>11</v>
+      </c>
+      <c r="I7">
+        <v>15</v>
+      </c>
+      <c r="J7">
         <v>8</v>
       </c>
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-      <c r="E7">
-        <v>3</v>
-      </c>
-      <c r="F7">
-        <v>6</v>
-      </c>
-      <c r="G7">
-        <v>7</v>
-      </c>
-      <c r="H7">
-        <v>6</v>
-      </c>
-      <c r="I7">
-        <v>5</v>
-      </c>
-      <c r="J7">
-        <v>2</v>
-      </c>
       <c r="K7">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="M7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>11</v>
-      </c>
-      <c r="C8">
-        <v>12</v>
-      </c>
-      <c r="D8">
-        <v>25</v>
-      </c>
-      <c r="E8">
-        <v>19</v>
-      </c>
-      <c r="F8">
-        <v>33</v>
-      </c>
-      <c r="G8">
-        <v>14</v>
-      </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8">
-        <v>17</v>
-      </c>
-      <c r="J8">
-        <v>16</v>
-      </c>
-      <c r="K8">
-        <v>11</v>
-      </c>
-      <c r="L8">
-        <v>9</v>
-      </c>
-      <c r="M8">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>17</v>
-      </c>
-      <c r="C9">
-        <v>14</v>
-      </c>
-      <c r="D9">
-        <v>32</v>
-      </c>
-      <c r="E9">
-        <v>23</v>
-      </c>
-      <c r="F9">
-        <v>40</v>
-      </c>
-      <c r="G9">
-        <v>24</v>
-      </c>
-      <c r="H9">
-        <v>16</v>
-      </c>
-      <c r="I9">
-        <v>26</v>
-      </c>
-      <c r="J9">
-        <v>19</v>
-      </c>
-      <c r="K9">
-        <v>18</v>
-      </c>
-      <c r="L9">
-        <v>17</v>
-      </c>
-      <c r="M9">
         <v>16</v>
       </c>
     </row>

</xml_diff>